<commit_message>
maj courbe survie + icdo
</commit_message>
<xml_diff>
--- a/ICDO.xlsx
+++ b/ICDO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20389"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\medical-srv1\labo-hemato\RRHMBN\RAPPORTS_ACTIVITE\Rap-Acti2024\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\medical-srv1\labo-hemato\RRHMBN\RAPPORTS_ACTIVITE\Rap-Acti2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7422D9D-8D60-4917-9DA5-F68744153A28}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F60C8DEF-4662-4C57-9C36-F378500013F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27765" yWindow="3780" windowWidth="30525" windowHeight="17535" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="15" windowWidth="28065" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="icdo" sheetId="1" r:id="rId1"/>
@@ -21,9 +21,9 @@
     <externalReference r:id="rId4"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">icdo!$A$1:$XFC$184</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">icdo!$A$1:$XFC$185</definedName>
     <definedName name="adicap">[1]adicap!$A$1:$B$515</definedName>
-    <definedName name="icdo">icdo!$A$1:$I$184</definedName>
+    <definedName name="icdo">icdo!$A$1:$I$185</definedName>
     <definedName name="id">#REF!</definedName>
     <definedName name="idhem">#REF!</definedName>
     <definedName name="idp">#REF!</definedName>
@@ -33,7 +33,7 @@
     <definedName name="xcir1" hidden="1">-3.14159265358979+(ROW(OFFSET(#REF!,0,0,500,1))-1)*0.0125915537218028</definedName>
     <definedName name="xdata1" hidden="1">-6000+(ROW(OFFSET(#REF!,0,0,1000,1))-1)*7.00700700700701</definedName>
     <definedName name="xdata2" hidden="1">0+(ROW(OFFSET(#REF!,0,0,1000,1))-1)*0.12012012012012</definedName>
-    <definedName name="xt_label">xt!$A$1:$B$162</definedName>
+    <definedName name="xt_label">xt!$A$1:$B$184</definedName>
     <definedName name="ycir1" hidden="1">1*COS([0]!xcir1)+0</definedName>
     <definedName name="ydata1" hidden="1">[2]!XLSTAT_PDFNormal([0]!xdata1,62.7394404089321,46.7064870962644)</definedName>
     <definedName name="ydata2" hidden="1">[2]!XLSTAT_PDFNormal([0]!xdata2,68.8138116154223,17.56618401385)</definedName>
@@ -43,6 +43,20 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -54,7 +68,7 @@
     <author>CORNET EDOUARD</author>
   </authors>
   <commentList>
-    <comment ref="C86" authorId="0" shapeId="0" xr:uid="{ADECF2B6-4C9B-41F3-B7F3-2717A42BB90B}">
+    <comment ref="C87" authorId="0" shapeId="0" xr:uid="{ADECF2B6-4C9B-41F3-B7F3-2717A42BB90B}">
       <text>
         <r>
           <rPr>
@@ -78,7 +92,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C87" authorId="0" shapeId="0" xr:uid="{A75CE0F6-A0C4-437D-BF80-CB3CDF2F2BFC}">
+    <comment ref="C88" authorId="0" shapeId="0" xr:uid="{A75CE0F6-A0C4-437D-BF80-CB3CDF2F2BFC}">
       <text>
         <r>
           <rPr>
@@ -107,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1290" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1319" uniqueCount="452">
   <si>
     <t>ICD-O-3</t>
   </si>
@@ -1129,9 +1143,6 @@
     <t>Lymphoproliferative disorder, NOS</t>
   </si>
   <si>
-    <t>99711*</t>
-  </si>
-  <si>
     <t>Plasmacytic hyperplasia</t>
   </si>
   <si>
@@ -1460,6 +1471,12 @@
   </si>
   <si>
     <t>36: Néoplasie myéloïde/lymphoïde avec éosinophilie</t>
+  </si>
+  <si>
+    <t>Erdheim-Chester disease</t>
+  </si>
+  <si>
+    <t>Autre hémopathie (/1) - Non classé</t>
   </si>
 </sst>
 </file>
@@ -1681,7 +1698,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="adicap"/>
@@ -1696,7 +1713,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="XLSTAT"/>
@@ -1976,7 +1993,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:XFC184"/>
+  <dimension ref="A1:XFC185"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.85546875" style="1" customWidth="1"/>
@@ -2022,10 +2039,10 @@
         <v>8</v>
       </c>
       <c r="J1" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="K1" s="6" t="s">
         <v>395</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>396</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>9</v>
@@ -2078,9 +2095,9 @@
         <v>11</v>
       </c>
       <c r="J3" s="2"/>
-      <c r="K3" s="1" t="e">
+      <c r="K3" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -2088,13 +2105,13 @@
         <v>97091</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="F4" s="1">
         <v>104</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="H4" s="1">
         <v>100</v>
@@ -2102,9 +2119,9 @@
       <c r="I4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="1" t="e">
+      <c r="K4" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -2127,7 +2144,7 @@
         <v>104</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="H5" s="1">
         <v>100</v>
@@ -2135,9 +2152,9 @@
       <c r="I5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="1" t="e">
+      <c r="K5" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -2160,7 +2177,7 @@
         <v>110</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="H6" s="1">
         <v>100</v>
@@ -2168,9 +2185,9 @@
       <c r="I6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K6" s="1" t="e">
+      <c r="K6" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -2178,16 +2195,16 @@
         <v>97411</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F7" s="1">
         <v>108</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="H7" s="1">
         <v>100</v>
@@ -2195,9 +2212,9 @@
       <c r="I7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K7" s="1" t="e">
+      <c r="K7" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -2228,9 +2245,9 @@
       <c r="I8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="1" t="e">
+      <c r="K8" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
       <c r="L8" s="1" t="s">
         <v>203</v>
@@ -2258,9 +2275,9 @@
       <c r="I9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K9" s="1" t="e">
+      <c r="K9" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -2291,9 +2308,9 @@
       <c r="I10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K10" s="1" t="e">
+      <c r="K10" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -2319,9 +2336,9 @@
         <v>11</v>
       </c>
       <c r="J11" s="2"/>
-      <c r="K11" s="1" t="e">
+      <c r="K11" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -2332,7 +2349,7 @@
         <v>248</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F12" s="1">
         <v>102</v>
@@ -2371,7 +2388,7 @@
         <v>109</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="H13" s="1">
         <v>100</v>
@@ -2380,9 +2397,9 @@
         <v>11</v>
       </c>
       <c r="J13" s="2"/>
-      <c r="K13" s="1" t="e">
+      <c r="K13" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -2405,7 +2422,7 @@
         <v>104</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="H14" s="1">
         <v>100</v>
@@ -2413,9 +2430,9 @@
       <c r="I14" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K14" s="1" t="e">
+      <c r="K14" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -2423,22 +2440,22 @@
         <v>99711</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>31</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>344</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>345</v>
       </c>
       <c r="F15" s="1">
         <v>104</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="H15" s="1">
         <v>100</v>
@@ -2446,9 +2463,9 @@
       <c r="I15" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K15" s="1" t="e">
+      <c r="K15" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -2594,7 +2611,7 @@
         <v>105</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="H20" s="1">
         <v>100</v>
@@ -2603,12 +2620,12 @@
         <v>11</v>
       </c>
       <c r="J20" s="6"/>
-      <c r="K20" s="1" t="e">
+      <c r="K20" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
@@ -2639,9 +2656,9 @@
       <c r="I21" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K21" s="1" t="e">
+      <c r="K21" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
@@ -2718,13 +2735,13 @@
         <v>205</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F24" s="1">
         <v>306</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="H24" s="1">
         <v>300</v>
@@ -2737,7 +2754,7 @@
         <v>Granulomatose lymphomatoïde grade 3</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
@@ -2745,13 +2762,13 @@
         <v>99713</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F25" s="1">
         <v>305</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="H25" s="1">
         <v>300</v>
@@ -2864,7 +2881,7 @@
         <v>Leucémie aiguë de lignée ambiguë</v>
       </c>
       <c r="L28" s="6" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
@@ -3295,10 +3312,10 @@
         <v>98783</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F42" s="1">
         <v>31</v>
@@ -3322,10 +3339,10 @@
         <v>98793</v>
       </c>
       <c r="B43" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="C43" s="1" t="s">
         <v>372</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>373</v>
       </c>
       <c r="F43" s="1">
         <v>31</v>
@@ -3580,7 +3597,7 @@
         <v>99123</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>269</v>
@@ -3676,16 +3693,16 @@
         <v>99843</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>56</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F54" s="1">
         <v>31</v>
@@ -3743,7 +3760,7 @@
         <v>99873</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>56</v>
@@ -4345,7 +4362,7 @@
         <v>98193</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C73" s="6"/>
       <c r="F73" s="1">
@@ -4365,7 +4382,7 @@
         <v>Leucémie aiguë lymphoblastique B</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.25">
@@ -13697,14 +13714,14 @@
         <v>96951</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C109" s="6"/>
       <c r="F109" s="1">
         <v>104</v>
       </c>
       <c r="G109" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="H109" s="1">
         <v>100</v>
@@ -13712,12 +13729,12 @@
       <c r="I109" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K109" s="1" t="e">
+      <c r="K109" s="1" t="str">
         <f t="shared" si="3"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
       <c r="L109" s="6" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.25">
@@ -14088,10 +14105,10 @@
         <v>97153</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F121" s="1">
         <v>27</v>
@@ -14250,7 +14267,7 @@
         <v>248</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F126" s="1">
         <v>27</v>
@@ -14376,7 +14393,7 @@
         <v>155</v>
       </c>
       <c r="C130" s="6" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F130" s="1">
         <v>29</v>
@@ -15165,28 +15182,28 @@
         <v>99803</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D154" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="E154" s="1" t="s">
         <v>349</v>
-      </c>
-      <c r="E154" s="1" t="s">
-        <v>350</v>
       </c>
       <c r="F154" s="1">
         <v>6</v>
       </c>
       <c r="G154" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H154" s="1">
         <v>6</v>
       </c>
       <c r="I154" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="J154" s="3"/>
       <c r="K154" s="1" t="str">
@@ -15199,28 +15216,28 @@
         <v>99823</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D155" s="1" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E155" s="1" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="F155" s="1">
         <v>6</v>
       </c>
       <c r="G155" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H155" s="1">
         <v>6</v>
       </c>
       <c r="I155" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="J155" s="3"/>
       <c r="K155" s="1" t="str">
@@ -15233,28 +15250,28 @@
         <v>99833</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C156" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D156" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="E156" s="1" t="s">
         <v>355</v>
-      </c>
-      <c r="E156" s="1" t="s">
-        <v>356</v>
       </c>
       <c r="F156" s="1">
         <v>6</v>
       </c>
       <c r="G156" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H156" s="1">
         <v>6</v>
       </c>
       <c r="I156" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="J156" s="3"/>
       <c r="K156" s="1" t="str">
@@ -15267,13 +15284,13 @@
         <v>99853</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D157" s="1" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E157" s="1" t="s">
         <v>299</v>
@@ -15282,13 +15299,13 @@
         <v>6</v>
       </c>
       <c r="G157" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H157" s="1">
         <v>6</v>
       </c>
       <c r="I157" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="J157" s="3"/>
       <c r="K157" s="1" t="str">
@@ -15301,13 +15318,13 @@
         <v>99863</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D158" s="1" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E158" s="1" t="s">
         <v>299</v>
@@ -15316,13 +15333,13 @@
         <v>6</v>
       </c>
       <c r="G158" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H158" s="1">
         <v>6</v>
       </c>
       <c r="I158" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="J158" s="3"/>
       <c r="K158" s="1" t="str">
@@ -15335,28 +15352,28 @@
         <v>99893</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D159" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="E159" s="1" t="s">
         <v>364</v>
-      </c>
-      <c r="E159" s="1" t="s">
-        <v>365</v>
       </c>
       <c r="F159" s="1">
         <v>6</v>
       </c>
       <c r="G159" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H159" s="1">
         <v>6</v>
       </c>
       <c r="I159" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="J159" s="3"/>
       <c r="K159" s="1" t="str">
@@ -15369,28 +15386,28 @@
         <v>99913</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>31</v>
       </c>
       <c r="D160" s="1" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E160" s="1" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F160" s="1">
         <v>6</v>
       </c>
       <c r="G160" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H160" s="1">
         <v>6</v>
       </c>
       <c r="I160" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="J160" s="3"/>
       <c r="K160" s="1" t="str">
@@ -15403,28 +15420,28 @@
         <v>99923</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>31</v>
       </c>
       <c r="D161" s="1" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E161" s="1" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F161" s="1">
         <v>6</v>
       </c>
       <c r="G161" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H161" s="1">
         <v>6</v>
       </c>
       <c r="I161" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="J161" s="3"/>
       <c r="K161" s="1" t="str">
@@ -15437,26 +15454,26 @@
         <v>99933</v>
       </c>
       <c r="B162" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="C162" s="1" t="s">
         <v>369</v>
-      </c>
-      <c r="C162" s="1" t="s">
-        <v>370</v>
       </c>
       <c r="F162" s="1">
         <v>6</v>
       </c>
       <c r="G162" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H162" s="1">
         <v>6</v>
       </c>
       <c r="I162" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="J162" s="3"/>
       <c r="K162" s="1" t="str">
-        <f t="shared" ref="K162:K184" si="5">VLOOKUP(A162,xt_label,2,FALSE)</f>
+        <f t="shared" ref="K162:K185" si="5">VLOOKUP(A162,xt_label,2,FALSE)</f>
         <v>Syndrome myélodysplasique (SMD)</v>
       </c>
     </row>
@@ -15567,7 +15584,7 @@
         <v>99753</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>31</v>
@@ -15862,19 +15879,10 @@
     </row>
     <row r="175" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A175" s="1">
-        <v>97563</v>
-      </c>
-      <c r="B175" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="C175" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D175" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="E175" s="1" t="s">
-        <v>139</v>
+        <v>97493</v>
+      </c>
+      <c r="B175" s="6" t="s">
+        <v>450</v>
       </c>
       <c r="F175" s="1">
         <v>301</v>
@@ -15895,10 +15903,10 @@
     </row>
     <row r="176" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A176" s="1">
-        <v>97573</v>
+        <v>97563</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C176" s="1" t="s">
         <v>29</v>
@@ -15928,13 +15936,13 @@
     </row>
     <row r="177" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A177" s="1">
-        <v>97593</v>
+        <v>97573</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C177" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D177" s="1" t="s">
         <v>134</v>
@@ -15961,31 +15969,43 @@
     </row>
     <row r="178" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A178" s="1">
-        <v>97661</v>
+        <v>97593</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>205</v>
+        <v>188</v>
       </c>
       <c r="C178" s="1" t="s">
-        <v>128</v>
+        <v>31</v>
       </c>
       <c r="D178" s="1" t="s">
-        <v>206</v>
+        <v>134</v>
       </c>
       <c r="E178" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="K178" s="1" t="e">
+        <v>139</v>
+      </c>
+      <c r="F178" s="1">
+        <v>301</v>
+      </c>
+      <c r="G178" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H178" s="1">
+        <v>300</v>
+      </c>
+      <c r="I178" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K178" s="1" t="str">
         <f t="shared" si="5"/>
-        <v>#N/A</v>
+        <v>Histiocytose maligne</v>
       </c>
     </row>
     <row r="179" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A179" s="1">
-        <v>97671</v>
+        <v>97661</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C179" s="1" t="s">
         <v>128</v>
@@ -15996,17 +16016,29 @@
       <c r="E179" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="K179" s="1" t="e">
+      <c r="F179" s="1">
+        <v>199</v>
+      </c>
+      <c r="G179" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="H179" s="1">
+        <v>100</v>
+      </c>
+      <c r="I179" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K179" s="1" t="str">
         <f t="shared" si="5"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="180" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A180" s="1">
-        <v>97681</v>
+        <v>97671</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C180" s="1" t="s">
         <v>128</v>
@@ -16017,51 +16049,62 @@
       <c r="E180" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="K180" s="1" t="e">
+      <c r="F180" s="1">
+        <v>199</v>
+      </c>
+      <c r="G180" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="H180" s="1">
+        <v>100</v>
+      </c>
+      <c r="I180" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K180" s="1" t="str">
         <f t="shared" si="5"/>
-        <v>#N/A</v>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="181" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A181" s="1">
-        <v>99653</v>
+        <v>97681</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>336</v>
+        <v>209</v>
       </c>
       <c r="C181" s="1" t="s">
-        <v>31</v>
+        <v>128</v>
       </c>
       <c r="D181" s="1" t="s">
-        <v>301</v>
+        <v>206</v>
       </c>
       <c r="E181" s="1" t="s">
-        <v>302</v>
+        <v>207</v>
       </c>
       <c r="F181" s="1">
-        <v>42</v>
-      </c>
-      <c r="G181" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="H181" s="2">
-        <v>4</v>
-      </c>
-      <c r="I181" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="J181" s="2"/>
+        <v>199</v>
+      </c>
+      <c r="G181" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="H181" s="1">
+        <v>100</v>
+      </c>
+      <c r="I181" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="K181" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Néoplasie myéloïde/lymphoïde avec éosinophilie</v>
+        <f>VLOOKUP(A181,xt_label,2,FALSE)</f>
+        <v>Autre hémopathie (/1)</v>
       </c>
     </row>
     <row r="182" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A182" s="1">
-        <v>99663</v>
+        <v>99653</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C182" s="1" t="s">
         <v>31</v>
@@ -16092,10 +16135,10 @@
     </row>
     <row r="183" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A183" s="1">
-        <v>99673</v>
+        <v>99663</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C183" s="1" t="s">
         <v>31</v>
@@ -16125,38 +16168,84 @@
       </c>
     </row>
     <row r="184" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A184" s="1" t="s">
+      <c r="A184" s="1">
+        <v>99673</v>
+      </c>
+      <c r="B184" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C184" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D184" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="E184" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="F184" s="1">
+        <v>42</v>
+      </c>
+      <c r="G184" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="H184" s="2">
+        <v>4</v>
+      </c>
+      <c r="I184" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="J184" s="2"/>
+      <c r="K184" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Néoplasie myéloïde/lymphoïde avec éosinophilie</v>
+      </c>
+    </row>
+    <row r="185" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A185" s="1">
+        <v>99711</v>
+      </c>
+      <c r="B185" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="B184" s="1" t="s">
+      <c r="C185" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D185" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="E185" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="F185" s="1">
+        <v>199</v>
+      </c>
+      <c r="G185" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="H185" s="1">
+        <v>100</v>
+      </c>
+      <c r="I185" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K185" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Autre hémopathie (/1)</v>
+      </c>
+      <c r="L185" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="C184" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D184" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="E184" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="K184" s="1" t="e">
-        <f t="shared" si="5"/>
-        <v>#N/A</v>
-      </c>
-      <c r="L184" s="1" t="s">
-        <v>342</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:XFC184" xr:uid="{3C71BD9C-CD8C-4616-B7D0-60D6CE2D4F98}"/>
+  <autoFilter ref="A1:XFC185" xr:uid="{3C71BD9C-CD8C-4616-B7D0-60D6CE2D4F98}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7F75522-822F-4A23-99F0-B9CA461B41C9}">
-  <dimension ref="A1:J162"/>
+  <dimension ref="A1:J184"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="63.5703125" bestFit="1" customWidth="1"/>
@@ -16194,7 +16283,7 @@
         <v>19</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16205,7 +16294,7 @@
         <v>19</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16216,7 +16305,7 @@
         <v>19</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16227,7 +16316,7 @@
         <v>16</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16238,7 +16327,7 @@
         <v>37</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16249,7 +16338,7 @@
         <v>37</v>
       </c>
       <c r="J9" s="11" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16260,7 +16349,7 @@
         <v>37</v>
       </c>
       <c r="J10" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16271,7 +16360,7 @@
         <v>37</v>
       </c>
       <c r="J11" s="11" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16282,7 +16371,7 @@
         <v>37</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16293,7 +16382,7 @@
         <v>37</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16304,7 +16393,7 @@
         <v>37</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16315,7 +16404,7 @@
         <v>37</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16326,7 +16415,7 @@
         <v>37</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16337,7 +16426,7 @@
         <v>37</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16348,7 +16437,7 @@
         <v>37</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16359,7 +16448,7 @@
         <v>37</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16370,7 +16459,7 @@
         <v>37</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16378,10 +16467,10 @@
         <v>96703</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16392,7 +16481,7 @@
         <v>72</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16403,7 +16492,7 @@
         <v>76</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16414,7 +16503,7 @@
         <v>19</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16425,7 +16514,7 @@
         <v>82</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16436,7 +16525,7 @@
         <v>82</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16447,7 +16536,7 @@
         <v>82</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16458,7 +16547,7 @@
         <v>82</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16466,13 +16555,13 @@
         <v>96873</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16483,7 +16572,7 @@
         <v>82</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16494,7 +16583,7 @@
         <v>96</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16505,7 +16594,7 @@
         <v>16</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16516,7 +16605,7 @@
         <v>16</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16527,7 +16616,7 @@
         <v>16</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16538,7 +16627,7 @@
         <v>16</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16549,7 +16638,7 @@
         <v>96</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16560,7 +16649,7 @@
         <v>110</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16571,7 +16660,7 @@
         <v>110</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16582,7 +16671,7 @@
         <v>110</v>
       </c>
       <c r="J39" s="12" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16694,10 +16783,10 @@
         <v>97273</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16705,10 +16794,10 @@
         <v>97283</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16716,7 +16805,7 @@
         <v>97293</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16724,7 +16813,7 @@
         <v>97313</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16732,7 +16821,7 @@
         <v>97323</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16740,7 +16829,7 @@
         <v>97333</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16748,7 +16837,7 @@
         <v>97343</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16756,7 +16845,7 @@
         <v>97353</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16780,7 +16869,7 @@
         <v>97403</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16788,7 +16877,7 @@
         <v>97413</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -16796,12 +16885,12 @@
         <v>97423</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="9">
-        <v>97503</v>
+        <v>97493</v>
       </c>
       <c r="B66" s="10" t="s">
         <v>172</v>
@@ -16809,7 +16898,7 @@
     </row>
     <row r="67" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="9">
-        <v>97513</v>
+        <v>97503</v>
       </c>
       <c r="B67" s="10" t="s">
         <v>172</v>
@@ -16817,7 +16906,7 @@
     </row>
     <row r="68" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="9">
-        <v>97543</v>
+        <v>97513</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>172</v>
@@ -16825,7 +16914,7 @@
     </row>
     <row r="69" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="9">
-        <v>97553</v>
+        <v>97543</v>
       </c>
       <c r="B69" s="10" t="s">
         <v>172</v>
@@ -16833,7 +16922,7 @@
     </row>
     <row r="70" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="9">
-        <v>97563</v>
+        <v>97553</v>
       </c>
       <c r="B70" s="10" t="s">
         <v>172</v>
@@ -16841,7 +16930,7 @@
     </row>
     <row r="71" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="9">
-        <v>97573</v>
+        <v>97563</v>
       </c>
       <c r="B71" s="10" t="s">
         <v>172</v>
@@ -16849,47 +16938,47 @@
     </row>
     <row r="72" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="9">
-        <v>97583</v>
+        <v>97573</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>403</v>
+        <v>172</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="9">
-        <v>97593</v>
+        <v>97583</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>172</v>
+        <v>402</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="9">
-        <v>97603</v>
+        <v>97593</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>191</v>
+        <v>172</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="9">
-        <v>97613</v>
+        <v>97603</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>72</v>
+        <v>191</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="9">
-        <v>97623</v>
+        <v>97613</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>191</v>
+        <v>72</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="9">
-        <v>97643</v>
+        <v>97623</v>
       </c>
       <c r="B77" s="10" t="s">
         <v>191</v>
@@ -16897,546 +16986,546 @@
     </row>
     <row r="78" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="9">
-        <v>97663</v>
+        <v>97643</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>383</v>
+        <v>191</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="9">
-        <v>97953</v>
+        <v>97663</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>16</v>
+        <v>382</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="9">
-        <v>98003</v>
+        <v>97953</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>404</v>
+        <v>16</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="9">
-        <v>98013</v>
+        <v>98003</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="82" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="9">
-        <v>98053</v>
+        <v>98013</v>
       </c>
       <c r="B82" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="C82" s="10" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
     </row>
     <row r="83" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="9">
-        <v>98063</v>
+        <v>98053</v>
       </c>
       <c r="B83" s="10" t="s">
         <v>223</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="84" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="9">
-        <v>98073</v>
+        <v>98063</v>
       </c>
       <c r="B84" s="10" t="s">
         <v>223</v>
       </c>
       <c r="C84" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="9">
-        <v>98083</v>
+        <v>98073</v>
       </c>
       <c r="B85" s="10" t="s">
         <v>223</v>
       </c>
       <c r="C85" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="86" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="9">
-        <v>98093</v>
+        <v>98083</v>
       </c>
       <c r="B86" s="10" t="s">
         <v>223</v>
       </c>
       <c r="C86" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="9">
-        <v>98113</v>
+        <v>98093</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>413</v>
+        <v>223</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="9">
-        <v>98123</v>
+        <v>98113</v>
       </c>
       <c r="B88" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C88" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="89" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="9">
-        <v>98133</v>
+        <v>98123</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C89" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="90" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="9">
-        <v>98143</v>
+        <v>98133</v>
       </c>
       <c r="B90" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C90" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="91" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="9">
-        <v>98153</v>
+        <v>98143</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C91" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="92" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="9">
-        <v>98163</v>
+        <v>98153</v>
       </c>
       <c r="B92" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C92" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="93" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="9">
-        <v>98173</v>
+        <v>98163</v>
       </c>
       <c r="B93" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C93" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="94" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="9">
-        <v>98183</v>
+        <v>98173</v>
       </c>
       <c r="B94" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C94" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="95" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" s="9">
-        <v>98193</v>
+        <v>98183</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C95" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="96" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A96" s="9">
-        <v>98203</v>
+        <v>98193</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>19</v>
+        <v>412</v>
+      </c>
+      <c r="C96" s="10" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="97" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" s="9">
-        <v>98233</v>
+        <v>98203</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>397</v>
+        <v>19</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="9">
-        <v>98263</v>
+        <v>98233</v>
       </c>
       <c r="B98" s="10" t="s">
-        <v>413</v>
-      </c>
-      <c r="C98" s="10" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="9">
-        <v>98273</v>
+        <v>98263</v>
       </c>
       <c r="B99" s="10" t="s">
-        <v>110</v>
+        <v>412</v>
+      </c>
+      <c r="C99" s="10" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A100" s="9">
-        <v>98311</v>
+        <v>98273</v>
       </c>
       <c r="B100" s="10" t="s">
-        <v>405</v>
+        <v>110</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A101" s="9">
-        <v>98313</v>
+        <v>98311</v>
       </c>
       <c r="B101" s="10" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="9">
-        <v>98323</v>
+        <v>98313</v>
       </c>
       <c r="B102" s="10" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="9">
-        <v>98333</v>
+        <v>98323</v>
       </c>
       <c r="B103" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="104" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="9">
-        <v>98343</v>
+        <v>98333</v>
       </c>
       <c r="B104" s="10" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="105" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" s="9">
-        <v>98353</v>
+        <v>98343</v>
       </c>
       <c r="B105" s="10" t="s">
-        <v>413</v>
-      </c>
-      <c r="C105" s="10" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
     </row>
     <row r="106" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A106" s="9">
-        <v>98363</v>
+        <v>98353</v>
       </c>
       <c r="B106" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C106" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="107" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A107" s="9">
-        <v>98373</v>
+        <v>98363</v>
       </c>
       <c r="B107" s="10" t="s">
-        <v>399</v>
+        <v>412</v>
+      </c>
+      <c r="C107" s="10" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="108" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A108" s="9">
-        <v>98403</v>
+        <v>98373</v>
       </c>
       <c r="B108" s="10" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
     </row>
     <row r="109" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" s="9">
-        <v>98603</v>
+        <v>98403</v>
       </c>
       <c r="B109" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="110" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="9">
-        <v>98613</v>
+        <v>98603</v>
       </c>
       <c r="B110" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" s="9">
-        <v>98633</v>
+        <v>98613</v>
       </c>
       <c r="B111" s="10" t="s">
-        <v>274</v>
+        <v>403</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A112" s="9">
-        <v>98653</v>
+        <v>98633</v>
       </c>
       <c r="B112" s="10" t="s">
-        <v>404</v>
+        <v>274</v>
       </c>
     </row>
     <row r="113" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" s="9">
-        <v>98663</v>
+        <v>98653</v>
       </c>
       <c r="B113" s="10" t="s">
-        <v>279</v>
+        <v>403</v>
       </c>
     </row>
     <row r="114" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A114" s="9">
-        <v>98673</v>
+        <v>98663</v>
       </c>
       <c r="B114" s="10" t="s">
-        <v>404</v>
+        <v>279</v>
       </c>
     </row>
     <row r="115" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A115" s="9">
-        <v>98693</v>
+        <v>98673</v>
       </c>
       <c r="B115" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="116" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" s="9">
-        <v>98703</v>
+        <v>98693</v>
       </c>
       <c r="B116" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A117" s="9">
-        <v>98713</v>
+        <v>98703</v>
       </c>
       <c r="B117" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A118" s="9">
-        <v>98723</v>
+        <v>98713</v>
       </c>
       <c r="B118" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="119" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A119" s="9">
-        <v>98733</v>
+        <v>98723</v>
       </c>
       <c r="B119" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="120" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A120" s="9">
-        <v>98743</v>
+        <v>98733</v>
       </c>
       <c r="B120" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A121" s="9">
-        <v>98753</v>
+        <v>98743</v>
       </c>
       <c r="B121" s="10" t="s">
-        <v>274</v>
+        <v>403</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A122" s="9">
-        <v>98763</v>
+        <v>98753</v>
       </c>
       <c r="B122" s="10" t="s">
-        <v>290</v>
+        <v>274</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" s="9">
-        <v>98773</v>
+        <v>98763</v>
       </c>
       <c r="B123" s="10" t="s">
-        <v>404</v>
+        <v>290</v>
       </c>
     </row>
     <row r="124" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A124" s="9">
-        <v>98783</v>
+        <v>98773</v>
       </c>
       <c r="B124" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="125" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A125" s="9">
-        <v>98793</v>
+        <v>98783</v>
       </c>
       <c r="B125" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="126" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A126" s="9">
-        <v>98913</v>
+        <v>98793</v>
       </c>
       <c r="B126" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="127" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A127" s="9">
-        <v>98953</v>
+        <v>98913</v>
       </c>
       <c r="B127" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="128" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="9">
-        <v>98963</v>
+        <v>98953</v>
       </c>
       <c r="B128" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="129" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A129" s="9">
-        <v>98973</v>
+        <v>98963</v>
       </c>
       <c r="B129" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="130" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A130" s="9">
-        <v>98983</v>
+        <v>98973</v>
       </c>
       <c r="B130" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A131" s="9">
-        <v>99103</v>
+        <v>98983</v>
       </c>
       <c r="B131" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="132" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A132" s="9">
-        <v>99113</v>
+        <v>99103</v>
       </c>
       <c r="B132" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="133" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A133" s="9">
-        <v>99123</v>
+        <v>99113</v>
       </c>
       <c r="B133" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="9">
-        <v>99203</v>
+        <v>99123</v>
       </c>
       <c r="B134" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="135" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A135" s="9">
-        <v>99303</v>
+        <v>99203</v>
       </c>
       <c r="B135" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="136" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A136" s="9">
-        <v>99313</v>
+        <v>99303</v>
       </c>
       <c r="B136" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="137" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A137" s="9">
-        <v>99403</v>
+        <v>99313</v>
       </c>
       <c r="B137" s="10" t="s">
-        <v>317</v>
+        <v>403</v>
       </c>
     </row>
     <row r="138" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A138" s="9">
-        <v>99453</v>
+        <v>99403</v>
       </c>
       <c r="B138" s="10" t="s">
-        <v>290</v>
+        <v>317</v>
       </c>
     </row>
     <row r="139" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A139" s="9">
-        <v>99463</v>
+        <v>99453</v>
       </c>
       <c r="B139" s="10" t="s">
         <v>290</v>
@@ -17444,55 +17533,55 @@
     </row>
     <row r="140" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A140" s="9">
-        <v>99483</v>
+        <v>99463</v>
       </c>
       <c r="B140" s="10" t="s">
-        <v>110</v>
+        <v>290</v>
       </c>
     </row>
     <row r="141" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A141" s="9">
-        <v>99503</v>
+        <v>99483</v>
       </c>
       <c r="B141" s="10" t="s">
-        <v>408</v>
+        <v>110</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A142" s="9">
-        <v>99603</v>
+        <v>99503</v>
       </c>
       <c r="B142" s="10" t="s">
-        <v>325</v>
+        <v>407</v>
       </c>
     </row>
     <row r="143" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A143" s="9">
-        <v>99613</v>
+        <v>99603</v>
       </c>
       <c r="B143" s="10" t="s">
-        <v>409</v>
+        <v>325</v>
       </c>
     </row>
     <row r="144" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A144" s="9">
-        <v>99623</v>
+        <v>99613</v>
       </c>
       <c r="B144" s="10" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A145" s="9">
-        <v>99633</v>
+        <v>99623</v>
       </c>
       <c r="B145" s="10" t="s">
-        <v>325</v>
+        <v>409</v>
       </c>
     </row>
     <row r="146" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A146" s="9">
-        <v>99643</v>
+        <v>99633</v>
       </c>
       <c r="B146" s="10" t="s">
         <v>325</v>
@@ -17500,131 +17589,295 @@
     </row>
     <row r="147" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A147" s="9">
-        <v>99653</v>
+        <v>99643</v>
       </c>
       <c r="B147" s="10" t="s">
-        <v>411</v>
+        <v>325</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A148" s="9">
-        <v>99663</v>
+        <v>99653</v>
       </c>
       <c r="B148" s="10" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A149" s="9">
-        <v>99673</v>
+        <v>99663</v>
       </c>
       <c r="B149" s="10" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A150" s="9">
-        <v>99713</v>
+        <v>99673</v>
       </c>
       <c r="B150" s="10" t="s">
-        <v>19</v>
+        <v>410</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A151" s="9">
-        <v>99753</v>
+        <v>99713</v>
       </c>
       <c r="B151" s="10" t="s">
-        <v>290</v>
+        <v>19</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A152" s="9">
-        <v>99803</v>
+        <v>99753</v>
       </c>
       <c r="B152" s="10" t="s">
-        <v>412</v>
+        <v>290</v>
       </c>
     </row>
     <row r="153" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A153" s="9">
-        <v>99823</v>
+        <v>99803</v>
       </c>
       <c r="B153" s="10" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A154" s="9">
-        <v>99833</v>
+        <v>99823</v>
       </c>
       <c r="B154" s="10" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A155" s="9">
-        <v>99843</v>
+        <v>99833</v>
       </c>
       <c r="B155" s="10" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
     </row>
     <row r="156" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A156" s="9">
-        <v>99853</v>
+        <v>99843</v>
       </c>
       <c r="B156" s="10" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
     </row>
     <row r="157" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A157" s="9">
-        <v>99863</v>
+        <v>99853</v>
       </c>
       <c r="B157" s="10" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="158" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A158" s="9">
-        <v>99873</v>
+        <v>99863</v>
       </c>
       <c r="B158" s="10" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="159" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A159" s="9">
-        <v>99893</v>
+        <v>99873</v>
       </c>
       <c r="B159" s="10" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="160" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A160" s="9">
-        <v>99913</v>
+        <v>99893</v>
       </c>
       <c r="B160" s="10" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="161" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A161" s="9">
-        <v>99923</v>
+        <v>99913</v>
       </c>
       <c r="B161" s="10" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="162" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A162" s="9">
+        <v>99923</v>
+      </c>
+      <c r="B162" s="10" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A163" s="9">
         <v>99933</v>
       </c>
-      <c r="B162" s="10" t="s">
-        <v>412</v>
-      </c>
+      <c r="B163" s="10" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A164" s="9">
+        <v>96951</v>
+      </c>
+      <c r="B164" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A165" s="9">
+        <v>97661</v>
+      </c>
+      <c r="B165" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A166" s="9">
+        <v>97671</v>
+      </c>
+      <c r="B166" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A167" s="9">
+        <v>97681</v>
+      </c>
+      <c r="B167" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A168" s="9">
+        <v>99711</v>
+      </c>
+      <c r="B168" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A169" s="9">
+        <v>95911</v>
+      </c>
+      <c r="B169" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A170" s="9">
+        <v>97091</v>
+      </c>
+      <c r="B170" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A171" s="9">
+        <v>97181</v>
+      </c>
+      <c r="B171" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A172" s="9">
+        <v>97401</v>
+      </c>
+      <c r="B172" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A173" s="9">
+        <v>97411</v>
+      </c>
+      <c r="B173" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A174" s="9">
+        <v>97651</v>
+      </c>
+      <c r="B174" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A175" s="9">
+        <v>97611</v>
+      </c>
+      <c r="B175" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A176" s="9">
+        <v>97691</v>
+      </c>
+      <c r="B176" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A177" s="9">
+        <v>98231</v>
+      </c>
+      <c r="B177" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A178" s="9">
+        <v>98981</v>
+      </c>
+      <c r="B178" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A179" s="9">
+        <v>99701</v>
+      </c>
+      <c r="B179" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A180" s="9">
+        <v>97521</v>
+      </c>
+      <c r="B180" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A181" s="9">
+        <v>97531</v>
+      </c>
+      <c r="B181" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A182" s="9"/>
+      <c r="B182" s="10"/>
+    </row>
+    <row r="183" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A183" s="9"/>
+      <c r="B183" s="10"/>
+    </row>
+    <row r="184" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A184" s="9"/>
+      <c r="B184" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>